<commit_message>
bee bee boo boo
</commit_message>
<xml_diff>
--- a/data/clean/AR_methods.xlsx
+++ b/data/clean/AR_methods.xlsx
@@ -5,15 +5,16 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\thema\OneDrive\Documents\dissertation\survey\github\data\clean\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bmcgreal\Documents\dissertation\survey\data\clean\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{42DE9070-D0DE-4C4A-A245-71664538A965}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{74E8B6D6-D4C1-424B-912C-3484823C32BD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="24240" windowHeight="13140" xr2:uid="{70F81E01-4849-42CD-AB9B-9414582B1355}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{70F81E01-4849-42CD-AB9B-9414582B1355}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Final" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -25,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="29">
   <si>
     <t>Chinook</t>
   </si>
@@ -103,6 +104,15 @@
   </si>
   <si>
     <t>Total redd counts * Fish per redd estimate + Dam counts</t>
+  </si>
+  <si>
+    <t>Survey Method</t>
+  </si>
+  <si>
+    <t>Species</t>
+  </si>
+  <si>
+    <t>Relative Bias</t>
   </si>
 </sst>
 </file>
@@ -144,9 +154,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -165,9 +176,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -205,7 +216,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -311,7 +322,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -453,7 +464,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -462,13 +473,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B32334F8-B11A-4935-8120-0620CA328AA2}">
   <dimension ref="A1:E30"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="10" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="75.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="75.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
       <c r="B1" t="s">
         <v>12</v>
       </c>
@@ -482,7 +493,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -499,7 +510,7 @@
         <v>3.22</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
       <c r="B3">
         <v>9</v>
       </c>
@@ -513,7 +524,7 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
       <c r="B4">
         <v>11</v>
       </c>
@@ -527,7 +538,7 @@
         <v>7.0000000000000007E-2</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
       <c r="B5">
         <v>16</v>
       </c>
@@ -541,7 +552,7 @@
         <v>0.4</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
       <c r="B6">
         <v>17</v>
       </c>
@@ -555,7 +566,7 @@
         <v>7.0000000000000007E-2</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
       <c r="B7">
         <v>18</v>
       </c>
@@ -569,7 +580,7 @@
         <v>0.35</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
       <c r="B8">
         <v>21</v>
       </c>
@@ -583,7 +594,7 @@
         <v>0.3</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
       <c r="B9">
         <v>22</v>
       </c>
@@ -597,7 +608,7 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
       <c r="B10">
         <v>29</v>
       </c>
@@ -611,7 +622,7 @@
         <v>0.06</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>14</v>
       </c>
@@ -628,7 +639,7 @@
         <v>0.63</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.35">
       <c r="B13">
         <v>2</v>
       </c>
@@ -642,7 +653,7 @@
         <v>1.04</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.35">
       <c r="B14">
         <v>3</v>
       </c>
@@ -656,7 +667,7 @@
         <v>0.59</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.35">
       <c r="B15">
         <v>4</v>
       </c>
@@ -670,7 +681,7 @@
         <v>0.3</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.35">
       <c r="B16">
         <v>7</v>
       </c>
@@ -684,7 +695,7 @@
         <v>0.42</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.35">
       <c r="B17">
         <v>8</v>
       </c>
@@ -698,7 +709,7 @@
         <v>0.43</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.35">
       <c r="B18">
         <v>9</v>
       </c>
@@ -712,7 +723,7 @@
         <v>0.32</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.35">
       <c r="B19">
         <v>10</v>
       </c>
@@ -726,7 +737,7 @@
         <v>0.18</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.35">
       <c r="B20">
         <v>11</v>
       </c>
@@ -740,7 +751,7 @@
         <v>1.22</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.35">
       <c r="B21">
         <v>19</v>
       </c>
@@ -754,7 +765,7 @@
         <v>0.31</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>22</v>
       </c>
@@ -771,7 +782,7 @@
         <v>0.06</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.35">
       <c r="B24">
         <v>11</v>
       </c>
@@ -785,7 +796,7 @@
         <v>0.02</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.35">
       <c r="B25">
         <v>14</v>
       </c>
@@ -799,7 +810,7 @@
         <v>0.08</v>
       </c>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.35">
       <c r="B26">
         <v>15</v>
       </c>
@@ -813,7 +824,7 @@
         <v>0.16</v>
       </c>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.35">
       <c r="B27">
         <v>16</v>
       </c>
@@ -827,7 +838,7 @@
         <v>0.06</v>
       </c>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.35">
       <c r="B28">
         <v>21</v>
       </c>
@@ -841,7 +852,7 @@
         <v>0.14000000000000001</v>
       </c>
     </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:5" x14ac:dyDescent="0.35">
       <c r="B29">
         <v>22</v>
       </c>
@@ -855,7 +866,7 @@
         <v>0.75</v>
       </c>
     </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.35">
       <c r="B30">
         <v>23</v>
       </c>
@@ -866,6 +877,341 @@
         <v>0.41</v>
       </c>
       <c r="E30">
+        <v>6.9999999999999999E-4</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8F66EEEC-6E47-4ABB-93FD-D263C298AAF2}">
+  <dimension ref="A1:D30"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="10" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="75.453125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.6328125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>27</v>
+      </c>
+      <c r="B1" t="s">
+        <v>26</v>
+      </c>
+      <c r="C1" t="s">
+        <v>28</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C2">
+        <v>-1.36</v>
+      </c>
+      <c r="D2">
+        <v>3.22</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="B3" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C3" s="2">
+        <v>0</v>
+      </c>
+      <c r="D3">
+        <v>0.12</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="B4" t="s">
+        <v>5</v>
+      </c>
+      <c r="C4">
+        <v>0.25</v>
+      </c>
+      <c r="D4">
+        <v>7.0000000000000007E-2</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="B5" t="s">
+        <v>6</v>
+      </c>
+      <c r="C5">
+        <v>0.85</v>
+      </c>
+      <c r="D5">
+        <v>0.4</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="B6" t="s">
+        <v>13</v>
+      </c>
+      <c r="C6">
+        <v>-7.0000000000000007E-2</v>
+      </c>
+      <c r="D6">
+        <v>7.0000000000000007E-2</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="B7" t="s">
+        <v>7</v>
+      </c>
+      <c r="C7">
+        <v>-1.98</v>
+      </c>
+      <c r="D7">
+        <v>0.35</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="B8" t="s">
+        <v>8</v>
+      </c>
+      <c r="C8">
+        <v>-0.13</v>
+      </c>
+      <c r="D8">
+        <v>0.3</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="B9" t="s">
+        <v>9</v>
+      </c>
+      <c r="C9">
+        <v>1.1599999999999999</v>
+      </c>
+      <c r="D9">
+        <v>0.12</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="B10" t="s">
+        <v>10</v>
+      </c>
+      <c r="C10">
+        <v>0.43</v>
+      </c>
+      <c r="D10">
+        <v>0.06</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A12" t="s">
+        <v>14</v>
+      </c>
+      <c r="B12" t="s">
+        <v>15</v>
+      </c>
+      <c r="C12">
+        <v>-0.63</v>
+      </c>
+      <c r="D12">
+        <v>0.63</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="B13" t="s">
+        <v>16</v>
+      </c>
+      <c r="C13">
+        <v>0.27</v>
+      </c>
+      <c r="D13">
+        <v>1.04</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="B14" t="s">
+        <v>11</v>
+      </c>
+      <c r="C14">
+        <v>0.49</v>
+      </c>
+      <c r="D14">
+        <v>0.59</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="B15" t="s">
+        <v>17</v>
+      </c>
+      <c r="C15">
+        <v>0.59</v>
+      </c>
+      <c r="D15">
+        <v>0.3</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="B16" t="s">
+        <v>18</v>
+      </c>
+      <c r="C16">
+        <v>0.3</v>
+      </c>
+      <c r="D16">
+        <v>0.42</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="B17" t="s">
+        <v>19</v>
+      </c>
+      <c r="C17">
+        <v>-0.6</v>
+      </c>
+      <c r="D17">
+        <v>0.43</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="B18" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C18" s="2">
+        <v>0</v>
+      </c>
+      <c r="D18">
+        <v>0.32</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="B19" t="s">
+        <v>20</v>
+      </c>
+      <c r="C19">
+        <v>-0.34</v>
+      </c>
+      <c r="D19">
+        <v>0.18</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="B20" t="s">
+        <v>5</v>
+      </c>
+      <c r="C20">
+        <v>0.56999999999999995</v>
+      </c>
+      <c r="D20">
+        <v>1.22</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="B21" t="s">
+        <v>21</v>
+      </c>
+      <c r="C21">
+        <v>0.55000000000000004</v>
+      </c>
+      <c r="D21">
+        <v>0.31</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A23" t="s">
+        <v>22</v>
+      </c>
+      <c r="B23" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C23" s="2">
+        <v>0</v>
+      </c>
+      <c r="D23">
+        <v>0.06</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="B24" t="s">
+        <v>5</v>
+      </c>
+      <c r="C24">
+        <v>0.84</v>
+      </c>
+      <c r="D24">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="B25" t="s">
+        <v>23</v>
+      </c>
+      <c r="C25">
+        <v>-0.93</v>
+      </c>
+      <c r="D25">
+        <v>0.08</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="B26" t="s">
+        <v>24</v>
+      </c>
+      <c r="C26">
+        <v>-7.0000000000000007E-2</v>
+      </c>
+      <c r="D26">
+        <v>0.16</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="B27" t="s">
+        <v>6</v>
+      </c>
+      <c r="C27">
+        <v>1.1599999999999999</v>
+      </c>
+      <c r="D27">
+        <v>0.06</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="B28" t="s">
+        <v>8</v>
+      </c>
+      <c r="C28">
+        <v>0.13</v>
+      </c>
+      <c r="D28">
+        <v>0.14000000000000001</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="B29" t="s">
+        <v>9</v>
+      </c>
+      <c r="C29">
+        <v>-0.13</v>
+      </c>
+      <c r="D29">
+        <v>0.75</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="B30" t="s">
+        <v>25</v>
+      </c>
+      <c r="C30">
+        <v>0.41</v>
+      </c>
+      <c r="D30">
         <v>6.9999999999999999E-4</v>
       </c>
     </row>

</xml_diff>